<commit_message>
Added table Isolators - Digital to database
</commit_message>
<xml_diff>
--- a/To Add v2/00 Things To Add.xlsx
+++ b/To Add v2/00 Things To Add.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\Danakil_KiCad_DB\To Add v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16277CF7-01D1-4491-9EAA-BD8E9F0B8096}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C435369-D01B-40A3-A6E6-F83F7D3A8EDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="219">
   <si>
     <t>Table Name</t>
   </si>
@@ -721,7 +721,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -849,7 +849,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -924,41 +924,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="14">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="10">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1070,22 +1040,22 @@
   </sortState>
   <tableColumns count="24">
     <tableColumn id="1" xr3:uid="{24CA07BC-B564-425C-A1C9-824F8759E630}" name="Table Name"/>
-    <tableColumn id="2" xr3:uid="{9F4A02A6-F5DB-4F3A-A421-70A80F651F79}" name="Part 1" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{9F4A02A6-F5DB-4F3A-A421-70A80F651F79}" name="Part 1" dataDxfId="9"/>
     <tableColumn id="3" xr3:uid="{00BD6BA4-1F12-4724-AE31-3694BB4C53B5}" name="Part 2"/>
     <tableColumn id="4" xr3:uid="{1CAAE1E4-7D4D-47D1-8B9A-27C7679E6199}" name="Part 3"/>
     <tableColumn id="5" xr3:uid="{037D0EDD-3927-40D7-AFD5-1044A7CAD438}" name="Part 4"/>
     <tableColumn id="6" xr3:uid="{48D64EC1-0CF4-4E4E-A6D0-E999EC133A13}" name="Part 5"/>
     <tableColumn id="7" xr3:uid="{DD2BE2A2-2EB3-44FA-8623-456D01EA63F6}" name="Part 6"/>
     <tableColumn id="8" xr3:uid="{40DC5E7D-06D0-4B47-8AE6-2C5D8310EC72}" name="Part 7"/>
-    <tableColumn id="9" xr3:uid="{FC0664F5-2F12-48A0-AAC9-0BCA6842B8AC}" name="Spreadsheet" dataDxfId="12"/>
+    <tableColumn id="9" xr3:uid="{FC0664F5-2F12-48A0-AAC9-0BCA6842B8AC}" name="Spreadsheet" dataDxfId="8"/>
     <tableColumn id="10" xr3:uid="{0317F941-13E4-4D2B-BEEE-7C26C454AD40}" name="SQL Database"/>
     <tableColumn id="11" xr3:uid="{8162CF8B-28D2-4781-897D-4EAD7F56A2E8}" name=".kicad_dbl"/>
-    <tableColumn id="28" xr3:uid="{71D029E6-3725-4F01-AFCF-D6BA4C6D42C1}" name="Spreadsheet " dataDxfId="11"/>
+    <tableColumn id="28" xr3:uid="{71D029E6-3725-4F01-AFCF-D6BA4C6D42C1}" name="Spreadsheet " dataDxfId="7"/>
     <tableColumn id="12" xr3:uid="{431C6373-8E7D-4666-BDE1-467A0F9E453B}" name="Symbol Library"/>
     <tableColumn id="13" xr3:uid="{2DA1FDCD-CF72-45A1-B1B4-6EF51DFD8E52}" name="Footprint Library"/>
     <tableColumn id="17" xr3:uid="{78B76DFF-BD9A-4D3C-AABA-D1B79F14BCCA}" name="Functionality Verified?"/>
     <tableColumn id="15" xr3:uid="{D1E24C39-AA98-4732-9662-847B76D8D595}" name="Priority"/>
-    <tableColumn id="16" xr3:uid="{FF2332B8-8FC6-47C4-8923-30A2E08CE14A}" name="Completion (%)" dataDxfId="10">
+    <tableColumn id="16" xr3:uid="{FF2332B8-8FC6-47C4-8923-30A2E08CE14A}" name="Completion (%)" dataDxfId="6">
       <calculatedColumnFormula>(COUNTIF(Table1[[#This Row],[Spreadsheet]:[Functionality Verified?]],"=TRUE")/7) * 100</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="18" xr3:uid="{58412161-1BDA-44F7-B739-C52F8C666368}" name="Eff pt 1">
@@ -1378,7 +1348,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:AE152"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="14.08984375" customWidth="1"/>
     <col min="4" max="4" width="27.54296875" style="9" bestFit="1" customWidth="1"/>
@@ -1403,17 +1373,17 @@
     <col min="32" max="32" width="12.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:31" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:31">
       <c r="I1"/>
       <c r="P1"/>
       <c r="S1"/>
     </row>
-    <row r="2" spans="2:31" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:31">
       <c r="I2"/>
       <c r="P2"/>
       <c r="S2"/>
     </row>
-    <row r="3" spans="2:31" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:31">
       <c r="B3" s="17" t="s">
         <v>48</v>
       </c>
@@ -1431,7 +1401,7 @@
       <c r="P3"/>
       <c r="S3"/>
     </row>
-    <row r="4" spans="2:31" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:31">
       <c r="B4" s="18"/>
       <c r="C4" s="25"/>
       <c r="D4" s="9" t="s">
@@ -1445,7 +1415,7 @@
       <c r="P4"/>
       <c r="S4"/>
     </row>
-    <row r="5" spans="2:31" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:31">
       <c r="B5" s="18"/>
       <c r="C5" s="25"/>
       <c r="D5" s="9" t="s">
@@ -1461,23 +1431,23 @@
       <c r="I5"/>
       <c r="P5" s="8">
         <f t="shared" ref="P5:V5" si="0">100*COUNTIF(P12:P9999,"=TRUE")/COUNTA(P12:P9999)</f>
-        <v>37.588652482269502</v>
+        <v>38.297872340425535</v>
       </c>
       <c r="Q5" s="8">
         <f t="shared" si="0"/>
-        <v>37.588652482269502</v>
+        <v>38.297872340425535</v>
       </c>
       <c r="R5" s="8">
         <f t="shared" si="0"/>
-        <v>37.588652482269502</v>
+        <v>38.297872340425535</v>
       </c>
       <c r="S5" s="8">
         <f t="shared" si="0"/>
-        <v>41.134751773049643</v>
+        <v>41.843971631205676</v>
       </c>
       <c r="T5" s="8">
         <f t="shared" si="0"/>
-        <v>45.390070921985817</v>
+        <v>46.099290780141843</v>
       </c>
       <c r="U5" s="8">
         <f t="shared" si="0"/>
@@ -1488,7 +1458,7 @@
         <v>28.368794326241133</v>
       </c>
     </row>
-    <row r="6" spans="2:31" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:31">
       <c r="B6" s="18"/>
       <c r="C6" s="25"/>
       <c r="D6" s="9" t="s">
@@ -1502,10 +1472,10 @@
       <c r="P6"/>
       <c r="S6">
         <f>COUNTIF(S12:S9999,"=TRUE")</f>
-        <v>58</v>
-      </c>
-    </row>
-    <row r="7" spans="2:31" x14ac:dyDescent="0.35">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="7" spans="2:31">
       <c r="B7" s="18"/>
       <c r="C7" s="26"/>
       <c r="D7" s="11" t="s">
@@ -1513,13 +1483,13 @@
       </c>
       <c r="E7" s="15">
         <f>(COUNTIF(P12:V10039,"=TRUE")/COUNTA(P12:V10039))*100</f>
-        <v>42.046605876393109</v>
+        <v>42.553191489361701</v>
       </c>
       <c r="I7"/>
       <c r="P7"/>
       <c r="S7"/>
     </row>
-    <row r="8" spans="2:31" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:31">
       <c r="B8" s="18"/>
       <c r="C8" s="27" t="s">
         <v>144</v>
@@ -1529,7 +1499,7 @@
       </c>
       <c r="E8" s="13">
         <f>P5</f>
-        <v>37.588652482269502</v>
+        <v>38.297872340425535</v>
       </c>
       <c r="I8"/>
       <c r="P8"/>
@@ -1538,7 +1508,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="2:31" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:31">
       <c r="B9" s="18"/>
       <c r="C9" s="28"/>
       <c r="D9" s="9" t="s">
@@ -1546,7 +1516,7 @@
       </c>
       <c r="E9" s="14">
         <f>Q5</f>
-        <v>37.588652482269502</v>
+        <v>38.297872340425535</v>
       </c>
       <c r="I9"/>
       <c r="P9"/>
@@ -1563,7 +1533,7 @@
       <c r="AD9" s="1"/>
       <c r="AE9" s="1"/>
     </row>
-    <row r="10" spans="2:31" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:31">
       <c r="B10" s="18"/>
       <c r="C10" s="29"/>
       <c r="D10" s="11" t="s">
@@ -1571,7 +1541,7 @@
       </c>
       <c r="E10" s="15">
         <f>R5</f>
-        <v>37.588652482269502</v>
+        <v>38.297872340425535</v>
       </c>
       <c r="I10" s="19" t="s">
         <v>8</v>
@@ -1604,7 +1574,7 @@
       <c r="AD10" s="21"/>
       <c r="AE10" s="21"/>
     </row>
-    <row r="11" spans="2:31" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:31">
       <c r="B11" s="18"/>
       <c r="C11" s="24" t="s">
         <v>13</v>
@@ -1614,7 +1584,7 @@
       </c>
       <c r="E11" s="13">
         <f>S5</f>
-        <v>41.134751773049643</v>
+        <v>41.843971631205676</v>
       </c>
       <c r="H11" t="s">
         <v>0</v>
@@ -1689,7 +1659,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="2:31" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:31">
       <c r="B12" s="18"/>
       <c r="C12" s="25"/>
       <c r="D12" s="9" t="s">
@@ -1697,7 +1667,7 @@
       </c>
       <c r="E12" s="14">
         <f>T5</f>
-        <v>45.390070921985817</v>
+        <v>46.099290780141843</v>
       </c>
       <c r="H12" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
@@ -1772,7 +1742,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="2:31" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:31">
       <c r="B13" s="18"/>
       <c r="C13" s="26"/>
       <c r="D13" s="11" t="s">
@@ -1810,8 +1780,8 @@
       <c r="U13" t="b">
         <v>1</v>
       </c>
-      <c r="V13" t="b">
-        <v>0</v>
+      <c r="V13" t="s">
+        <v>184</v>
       </c>
       <c r="W13">
         <v>3</v>
@@ -1849,7 +1819,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="2:31" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:31">
       <c r="B14" s="18"/>
       <c r="C14" s="24" t="s">
         <v>16</v>
@@ -1931,7 +1901,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="2:31" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:31">
       <c r="B15" s="18"/>
       <c r="C15" s="25"/>
       <c r="D15" s="16" t="s">
@@ -2011,14 +1981,14 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="2:31" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:31">
       <c r="C16" s="25"/>
       <c r="D16" s="9" t="s">
         <v>148</v>
       </c>
       <c r="E16" s="14" cm="1">
         <f t="array" ref="E16">SUM(IF(W12:W9999 &gt; 0,X12:X9999,0))/COUNTIF(W12:W9999,"&gt;0")</f>
-        <v>41.269841269841265</v>
+        <v>49.206349206349202</v>
       </c>
       <c r="H16" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
@@ -2090,7 +2060,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="3:31" x14ac:dyDescent="0.35">
+    <row r="17" spans="3:31">
       <c r="C17" s="25"/>
       <c r="D17" s="9" t="s">
         <v>150</v>
@@ -2110,32 +2080,32 @@
         <v>98</v>
       </c>
       <c r="P17" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S17" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U17" t="b">
         <v>1</v>
       </c>
-      <c r="V17" t="b">
-        <v>0</v>
+      <c r="V17" t="s">
+        <v>184</v>
       </c>
       <c r="W17">
         <v>2</v>
       </c>
       <c r="X17" s="6">
         <f>(COUNTIF(Table1[[#This Row],[Spreadsheet]:[Functionality Verified?]],"=TRUE")/7) * 100</f>
-        <v>14.285714285714285</v>
+        <v>85.714285714285708</v>
       </c>
       <c r="Y17" t="str">
         <f>IF(COUNTBLANK(Table1[[#This Row],[Part 2]])=0,_xlfn.CONCAT(Table1[[#This Row],[Part 1]]," - "),IF(COUNTBLANK(Table1[[#This Row],[Part 1]])=0,Table1[[#This Row],[Part 1]],""))</f>
@@ -2166,7 +2136,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="3:31" x14ac:dyDescent="0.35">
+    <row r="18" spans="3:31">
       <c r="D18" s="9" t="s">
         <v>178</v>
       </c>
@@ -2247,7 +2217,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="3:31" x14ac:dyDescent="0.35">
+    <row r="19" spans="3:31">
       <c r="H19" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Isolators - Optoisolator</v>
@@ -2315,7 +2285,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="3:31" x14ac:dyDescent="0.35">
+    <row r="20" spans="3:31">
       <c r="H20" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Sensors - Temperature - Digital</v>
@@ -2386,7 +2356,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="3:31" x14ac:dyDescent="0.35">
+    <row r="21" spans="3:31">
       <c r="H21" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Capacitors - Polarized</v>
@@ -2454,7 +2424,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="3:31" x14ac:dyDescent="0.35">
+    <row r="22" spans="3:31">
       <c r="H22" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Clock&amp;Timing - ICs - DDS</v>
@@ -2525,7 +2495,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="3:31" x14ac:dyDescent="0.35">
+    <row r="23" spans="3:31">
       <c r="H23" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Clock&amp;Timing - Oscillators  - Fixed - Ceramic Resonator</v>
@@ -2599,7 +2569,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="3:31" x14ac:dyDescent="0.35">
+    <row r="24" spans="3:31">
       <c r="H24" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Clock&amp;Timing - Oscillators  - Fixed - TCXO</v>
@@ -2673,7 +2643,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="3:31" x14ac:dyDescent="0.35">
+    <row r="25" spans="3:31">
       <c r="H25" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Clock&amp;Timing - Oscillators  - VCOs - VCO</v>
@@ -2681,7 +2651,7 @@
       <c r="I25" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="J25" s="30" t="s">
+      <c r="J25" t="s">
         <v>124</v>
       </c>
       <c r="K25" t="s">
@@ -2747,7 +2717,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="3:31" x14ac:dyDescent="0.35">
+    <row r="26" spans="3:31">
       <c r="H26" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Clock&amp;Timing - Oscillators  - VCOs - VCTCXO</v>
@@ -2776,10 +2746,10 @@
       <c r="S26" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="T26" s="30" t="b">
-        <v>1</v>
-      </c>
-      <c r="U26" s="30" t="b">
+      <c r="T26" t="b">
+        <v>1</v>
+      </c>
+      <c r="U26" t="b">
         <v>0</v>
       </c>
       <c r="V26" t="b">
@@ -2821,7 +2791,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="3:31" x14ac:dyDescent="0.35">
+    <row r="27" spans="3:31">
       <c r="H27" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Clock&amp;Timing - Oscillators  - VCOs - VCXO</v>
@@ -2895,7 +2865,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="3:31" x14ac:dyDescent="0.35">
+    <row r="28" spans="3:31">
       <c r="H28" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Connectors - Banana Jacks</v>
@@ -2963,7 +2933,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="3:31" x14ac:dyDescent="0.35">
+    <row r="29" spans="3:31">
       <c r="H29" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Connectors - Battery Holders - Coin Cell</v>
@@ -3034,7 +3004,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="3:31" x14ac:dyDescent="0.35">
+    <row r="30" spans="3:31">
       <c r="H30" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Connectors - Battery Holders - Cylindrical</v>
@@ -3105,7 +3075,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="3:31" x14ac:dyDescent="0.35">
+    <row r="31" spans="3:31">
       <c r="H31" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Connectors - Card Edge</v>
@@ -3173,7 +3143,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="3:31" x14ac:dyDescent="0.35">
+    <row r="32" spans="3:31">
       <c r="H32" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Connectors - Coaxial</v>
@@ -3241,7 +3211,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="33" spans="8:31">
       <c r="H33" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Connectors - D-Sub - Backshells</v>
@@ -3312,7 +3282,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="34" spans="8:31">
       <c r="H34" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Connectors - D-Sub - Hybrid - Female - Inline</v>
@@ -3389,7 +3359,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="35" spans="8:31">
       <c r="H35" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Connectors - D-Sub - Hybrid - Male - Inline</v>
@@ -3466,7 +3436,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="36" spans="8:31">
       <c r="H36" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Connectors - D-Sub - Standard - Female - Inline</v>
@@ -3543,7 +3513,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="37" spans="8:31">
       <c r="H37" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Connectors - D-Sub - Standard - Female - PCB Mount</v>
@@ -3620,7 +3590,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="38" spans="8:31">
       <c r="H38" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Connectors - D-Sub - Standard - Male - Inline</v>
@@ -3697,7 +3667,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="39" spans="8:31">
       <c r="H39" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Connectors - D-Sub - Standard - Male - PCB Mount</v>
@@ -3774,7 +3744,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="40" spans="8:31">
       <c r="H40" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Connectors - Flat Flex</v>
@@ -3842,7 +3812,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="41" spans="8:31">
       <c r="H41" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Connectors - Jumpers</v>
@@ -3910,7 +3880,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="42" spans="8:31">
       <c r="H42" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Connectors - Power Entry Modules</v>
@@ -3978,7 +3948,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="43" spans="8:31">
       <c r="H43" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Connectors - Screw Connectors</v>
@@ -4046,7 +4016,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="44" spans="8:31">
       <c r="H44" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Connectors - SD Card Socket</v>
@@ -4114,7 +4084,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="45" spans="8:31">
       <c r="H45" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Connectors - Terminal Blocks - Wire to Board</v>
@@ -4185,7 +4155,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="46" spans="8:31">
       <c r="H46" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Contacts - Banana Plugs</v>
@@ -4253,7 +4223,7 @@
         <v/>
       </c>
     </row>
-    <row r="47" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="47" spans="8:31">
       <c r="H47" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Contacts - Ferrules</v>
@@ -4321,7 +4291,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="48" spans="8:31">
       <c r="H48" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Contacts - Ring Terminals</v>
@@ -4389,7 +4359,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="49" spans="8:31">
       <c r="H49" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Discreet - Diodes - Standard</v>
@@ -4460,7 +4430,7 @@
         <v/>
       </c>
     </row>
-    <row r="50" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="50" spans="8:31">
       <c r="H50" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Discreet - Transistors - BJT - PNP</v>
@@ -4534,7 +4504,7 @@
         <v/>
       </c>
     </row>
-    <row r="51" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="51" spans="8:31">
       <c r="H51" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Discreet - Transistors - GaNFET</v>
@@ -4605,7 +4575,7 @@
         <v/>
       </c>
     </row>
-    <row r="52" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="52" spans="8:31">
       <c r="H52" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Discreet - Transistors - JFET</v>
@@ -4676,7 +4646,7 @@
         <v/>
       </c>
     </row>
-    <row r="53" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="53" spans="8:31">
       <c r="H53" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Discreet - Transistors - MOSFET</v>
@@ -4747,7 +4717,7 @@
         <v/>
       </c>
     </row>
-    <row r="54" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="54" spans="8:31">
       <c r="H54" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Discreet - Transistors - SiCFET</v>
@@ -4818,7 +4788,7 @@
         <v/>
       </c>
     </row>
-    <row r="55" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="55" spans="8:31">
       <c r="H55" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Analog - Comparator</v>
@@ -4889,7 +4859,7 @@
         <v/>
       </c>
     </row>
-    <row r="56" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="56" spans="8:31">
       <c r="H56" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Analog - DAC</v>
@@ -4960,7 +4930,7 @@
         <v/>
       </c>
     </row>
-    <row r="57" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="57" spans="8:31">
       <c r="H57" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Embedded - FPGA</v>
@@ -5031,7 +5001,7 @@
         <v/>
       </c>
     </row>
-    <row r="58" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="58" spans="8:31">
       <c r="H58" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Embedded - PolarFire - SOC</v>
@@ -5105,7 +5075,7 @@
         <v/>
       </c>
     </row>
-    <row r="59" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="59" spans="8:31">
       <c r="H59" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Interface  - Analog Switch</v>
@@ -5176,7 +5146,7 @@
         <v/>
       </c>
     </row>
-    <row r="60" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="60" spans="8:31">
       <c r="H60" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Interface  - Controller</v>
@@ -5247,7 +5217,7 @@
         <v/>
       </c>
     </row>
-    <row r="61" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="61" spans="8:31">
       <c r="H61" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Interface  - Deserializer</v>
@@ -5318,7 +5288,7 @@
         <v/>
       </c>
     </row>
-    <row r="62" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="62" spans="8:31">
       <c r="H62" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Interface  - Drivers</v>
@@ -5389,7 +5359,7 @@
         <v/>
       </c>
     </row>
-    <row r="63" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="63" spans="8:31">
       <c r="H63" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Interface  - IO Expander</v>
@@ -5460,7 +5430,7 @@
         <v/>
       </c>
     </row>
-    <row r="64" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="64" spans="8:31">
       <c r="H64" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Interface  - Recievers</v>
@@ -5531,7 +5501,7 @@
         <v/>
       </c>
     </row>
-    <row r="65" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="65" spans="8:31">
       <c r="H65" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Interface  - Serializer</v>
@@ -5602,7 +5572,7 @@
         <v/>
       </c>
     </row>
-    <row r="66" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="66" spans="8:31">
       <c r="H66" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Interface  - Trancievers</v>
@@ -5673,7 +5643,7 @@
         <v/>
       </c>
     </row>
-    <row r="67" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="67" spans="8:31">
       <c r="H67" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Interface  - UART</v>
@@ -5744,7 +5714,7 @@
         <v/>
       </c>
     </row>
-    <row r="68" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="68" spans="8:31">
       <c r="H68" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Logic - Comparator - Digital</v>
@@ -5818,7 +5788,7 @@
         <v/>
       </c>
     </row>
-    <row r="69" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="69" spans="8:31">
       <c r="H69" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Logic - Counter - Up</v>
@@ -5892,7 +5862,7 @@
         <v/>
       </c>
     </row>
-    <row r="70" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="70" spans="8:31">
       <c r="H70" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Logic - Counter - Up&amp;Down</v>
@@ -5966,7 +5936,7 @@
         <v/>
       </c>
     </row>
-    <row r="71" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="71" spans="8:31">
       <c r="H71" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Logic - Demultiplexer - Digital</v>
@@ -6040,7 +6010,7 @@
         <v/>
       </c>
     </row>
-    <row r="72" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="72" spans="8:31">
       <c r="H72" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Logic - Flip Flops</v>
@@ -6111,7 +6081,7 @@
         <v/>
       </c>
     </row>
-    <row r="73" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="73" spans="8:31">
       <c r="H73" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Logic - Gates</v>
@@ -6182,7 +6152,7 @@
         <v/>
       </c>
     </row>
-    <row r="74" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="74" spans="8:31">
       <c r="H74" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Logic - Latches</v>
@@ -6253,7 +6223,7 @@
         <v/>
       </c>
     </row>
-    <row r="75" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="75" spans="8:31">
       <c r="H75" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Logic - Level Shifters</v>
@@ -6324,7 +6294,7 @@
         <v/>
       </c>
     </row>
-    <row r="76" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="76" spans="8:31">
       <c r="H76" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Logic - Multiplexer - Digital</v>
@@ -6398,7 +6368,7 @@
         <v/>
       </c>
     </row>
-    <row r="77" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="77" spans="8:31">
       <c r="H77" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Logic - Multivibrators</v>
@@ -6469,7 +6439,7 @@
         <v/>
       </c>
     </row>
-    <row r="78" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="78" spans="8:31">
       <c r="H78" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Logic - Shift Registers - PISO</v>
@@ -6543,7 +6513,7 @@
         <v/>
       </c>
     </row>
-    <row r="79" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="79" spans="8:31">
       <c r="H79" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Logic - Shift Registers - SIPO</v>
@@ -6617,7 +6587,7 @@
         <v/>
       </c>
     </row>
-    <row r="80" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="80" spans="8:31">
       <c r="H80" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Logic - Switch - Digital</v>
@@ -6691,7 +6661,7 @@
         <v/>
       </c>
     </row>
-    <row r="81" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="81" spans="8:31">
       <c r="H81" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Logic - Translators</v>
@@ -6762,7 +6732,7 @@
         <v/>
       </c>
     </row>
-    <row r="82" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="82" spans="8:31">
       <c r="H82" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Memory - DRAM</v>
@@ -6833,7 +6803,7 @@
         <v/>
       </c>
     </row>
-    <row r="83" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="83" spans="8:31">
       <c r="H83" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Memory - EEPROM</v>
@@ -6904,7 +6874,7 @@
         <v/>
       </c>
     </row>
-    <row r="84" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="84" spans="8:31">
       <c r="H84" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Memory - FLASH</v>
@@ -6975,7 +6945,7 @@
         <v/>
       </c>
     </row>
-    <row r="85" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="85" spans="8:31">
       <c r="H85" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Memory - SD Card</v>
@@ -7046,7 +7016,7 @@
         <v/>
       </c>
     </row>
-    <row r="86" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="86" spans="8:31">
       <c r="H86" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Power - Gate Driver - Isolated</v>
@@ -7120,7 +7090,7 @@
         <v/>
       </c>
     </row>
-    <row r="87" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="87" spans="8:31">
       <c r="H87" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Power - Gate Driver - Non Isolated</v>
@@ -7194,7 +7164,7 @@
         <v/>
       </c>
     </row>
-    <row r="88" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="88" spans="8:31">
       <c r="H88" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Power - Half&amp;H Bridge</v>
@@ -7265,7 +7235,7 @@
         <v/>
       </c>
     </row>
-    <row r="89" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="89" spans="8:31">
       <c r="H89" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Power - Supply Sequencing</v>
@@ -7336,7 +7306,7 @@
         <v/>
       </c>
     </row>
-    <row r="90" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="90" spans="8:31">
       <c r="H90" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Power - Switching Controler</v>
@@ -7407,7 +7377,7 @@
         <v/>
       </c>
     </row>
-    <row r="91" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="91" spans="8:31">
       <c r="H91" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - RTCs</v>
@@ -7475,7 +7445,7 @@
         <v/>
       </c>
     </row>
-    <row r="92" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="92" spans="8:31">
       <c r="H92" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Inductors - Common Mode Choke</v>
@@ -7543,7 +7513,7 @@
         <v/>
       </c>
     </row>
-    <row r="93" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="93" spans="8:31">
       <c r="H93" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Isolators - Analog</v>
@@ -7611,7 +7581,7 @@
         <v/>
       </c>
     </row>
-    <row r="94" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="94" spans="8:31">
       <c r="H94" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>LEDs - RGB</v>
@@ -7679,7 +7649,7 @@
         <v/>
       </c>
     </row>
-    <row r="95" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="95" spans="8:31">
       <c r="H95" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Mechanical  - Heat Shrink</v>
@@ -7747,7 +7717,7 @@
         <v/>
       </c>
     </row>
-    <row r="96" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="96" spans="8:31">
       <c r="H96" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Mechanical  - Nuts</v>
@@ -7815,7 +7785,7 @@
         <v/>
       </c>
     </row>
-    <row r="97" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="97" spans="8:31">
       <c r="H97" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Mechanical  - Spacers</v>
@@ -7883,7 +7853,7 @@
         <v/>
       </c>
     </row>
-    <row r="98" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="98" spans="8:31">
       <c r="H98" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Mechanical  - Standoffs  - F_F</v>
@@ -7954,7 +7924,7 @@
         <v/>
       </c>
     </row>
-    <row r="99" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="99" spans="8:31">
       <c r="H99" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Mechanical  - Standoffs  - M_F</v>
@@ -8025,7 +7995,7 @@
         <v/>
       </c>
     </row>
-    <row r="100" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="100" spans="8:31">
       <c r="H100" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Protection - PolyFuses</v>
@@ -8093,7 +8063,7 @@
         <v/>
       </c>
     </row>
-    <row r="101" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="101" spans="8:31">
       <c r="H101" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>PSUs - Chasis Mount - AC-DC</v>
@@ -8164,7 +8134,7 @@
         <v/>
       </c>
     </row>
-    <row r="102" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="102" spans="8:31">
       <c r="H102" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>PSUs - Chasis Mount - DC-DC</v>
@@ -8235,7 +8205,7 @@
         <v/>
       </c>
     </row>
-    <row r="103" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="103" spans="8:31">
       <c r="H103" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>PSUs - PCB Mount - AC-DC</v>
@@ -8305,7 +8275,7 @@
         <v/>
       </c>
     </row>
-    <row r="104" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="104" spans="8:31">
       <c r="H104" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Resistors - Network</v>
@@ -8373,7 +8343,7 @@
         <v/>
       </c>
     </row>
-    <row r="105" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="105" spans="8:31">
       <c r="H105" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Resistors - Single - Through Hole</v>
@@ -8444,7 +8414,7 @@
         <v/>
       </c>
     </row>
-    <row r="106" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="106" spans="8:31">
       <c r="H106" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Sensors - Capacitance To Digital</v>
@@ -8512,7 +8482,7 @@
         <v/>
       </c>
     </row>
-    <row r="107" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="107" spans="8:31">
       <c r="H107" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Sensors - Humidity</v>
@@ -8580,7 +8550,7 @@
         <v/>
       </c>
     </row>
-    <row r="108" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="108" spans="8:31">
       <c r="H108" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Sensors - Temperature - RTDs</v>
@@ -8651,7 +8621,7 @@
         <v/>
       </c>
     </row>
-    <row r="109" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="109" spans="8:31">
       <c r="H109" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Sensors - Touch Sensor - Capacitive</v>
@@ -8722,7 +8692,7 @@
         <v/>
       </c>
     </row>
-    <row r="110" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="110" spans="8:31">
       <c r="H110" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Transformer - Power - Chasis Mount</v>
@@ -8793,7 +8763,7 @@
         <v/>
       </c>
     </row>
-    <row r="111" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="111" spans="8:31">
       <c r="H111" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Transformer - Power - PCB Mount</v>
@@ -8864,7 +8834,7 @@
         <v/>
       </c>
     </row>
-    <row r="112" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="112" spans="8:31">
       <c r="H112" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Voltage References - Misc</v>
@@ -8932,7 +8902,7 @@
         <v/>
       </c>
     </row>
-    <row r="113" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="113" spans="8:31">
       <c r="H113" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Cables - Premade</v>
@@ -9000,7 +8970,7 @@
         <v/>
       </c>
     </row>
-    <row r="114" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="114" spans="8:31">
       <c r="H114" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Capacitors - Unpolarized</v>
@@ -9068,7 +9038,7 @@
         <v/>
       </c>
     </row>
-    <row r="115" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="115" spans="8:31">
       <c r="H115" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Clock&amp;Timing - ICs - Generators &amp; Synthisizers</v>
@@ -9139,7 +9109,7 @@
         <v/>
       </c>
     </row>
-    <row r="116" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="116" spans="8:31">
       <c r="H116" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Clock&amp;Timing - Oscillators  - Fixed - XO</v>
@@ -9213,7 +9183,7 @@
         <v/>
       </c>
     </row>
-    <row r="117" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="117" spans="8:31">
       <c r="H117" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Connectors - Barrel Jack</v>
@@ -9281,7 +9251,7 @@
         <v/>
       </c>
     </row>
-    <row r="118" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="118" spans="8:31">
       <c r="H118" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Connectors - IC socket</v>
@@ -9349,7 +9319,7 @@
         <v/>
       </c>
     </row>
-    <row r="119" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="119" spans="8:31">
       <c r="H119" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Connectors - Mezzanine</v>
@@ -9417,7 +9387,7 @@
         <v/>
       </c>
     </row>
-    <row r="120" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="120" spans="8:31">
       <c r="H120" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Connectors - Pads - SMD</v>
@@ -9488,7 +9458,7 @@
         <v/>
       </c>
     </row>
-    <row r="121" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="121" spans="8:31">
       <c r="H121" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Connectors - Pads - Through Hole</v>
@@ -9559,7 +9529,7 @@
         <v/>
       </c>
     </row>
-    <row r="122" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="122" spans="8:31">
       <c r="H122" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Connectors - Programming</v>
@@ -9627,7 +9597,7 @@
         <v/>
       </c>
     </row>
-    <row r="123" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="123" spans="8:31">
       <c r="H123" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Connectors - Rectangular</v>
@@ -9695,7 +9665,7 @@
         <v/>
       </c>
     </row>
-    <row r="124" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="124" spans="8:31">
       <c r="H124" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Connectors - RJ</v>
@@ -9763,7 +9733,7 @@
         <v/>
       </c>
     </row>
-    <row r="125" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="125" spans="8:31">
       <c r="H125" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Connectors - USB</v>
@@ -9831,7 +9801,7 @@
         <v/>
       </c>
     </row>
-    <row r="126" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="126" spans="8:31">
       <c r="H126" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Discreet - Diodes - Schottky</v>
@@ -9902,7 +9872,7 @@
         <v/>
       </c>
     </row>
-    <row r="127" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="127" spans="8:31">
       <c r="H127" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Discreet - Transistors - BJT - NPN</v>
@@ -9976,7 +9946,7 @@
         <v/>
       </c>
     </row>
-    <row r="128" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="128" spans="8:31">
       <c r="H128" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Analog - OP Amp</v>
@@ -10047,7 +10017,7 @@
         <v/>
       </c>
     </row>
-    <row r="129" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="129" spans="8:31">
       <c r="H129" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Embedded - MCU</v>
@@ -10118,7 +10088,7 @@
         <v/>
       </c>
     </row>
-    <row r="130" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="130" spans="8:31">
       <c r="H130" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Embedded - MCU - Module</v>
@@ -10192,7 +10162,7 @@
         <v/>
       </c>
     </row>
-    <row r="131" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="131" spans="8:31">
       <c r="H131" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Power - Ideal Diodes</v>
@@ -10263,7 +10233,7 @@
         <v/>
       </c>
     </row>
-    <row r="132" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="132" spans="8:31">
       <c r="H132" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>ICs - Power - Linear Regulation</v>
@@ -10334,7 +10304,7 @@
         <v/>
       </c>
     </row>
-    <row r="133" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="133" spans="8:31">
       <c r="H133" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Inductors</v>
@@ -10399,7 +10369,7 @@
         <v/>
       </c>
     </row>
-    <row r="134" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="134" spans="8:31">
       <c r="H134" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Inductors - Ferrite Bead</v>
@@ -10467,7 +10437,7 @@
         <v/>
       </c>
     </row>
-    <row r="135" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="135" spans="8:31">
       <c r="H135" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>LEDs - Standard - Indicator - SMD</v>
@@ -10541,7 +10511,7 @@
         <v/>
       </c>
     </row>
-    <row r="136" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="136" spans="8:31">
       <c r="H136" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>LEDs - Standard - Indicator - Through Hole</v>
@@ -10615,7 +10585,7 @@
         <v/>
       </c>
     </row>
-    <row r="137" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="137" spans="8:31">
       <c r="H137" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Mechanical  - Feet</v>
@@ -10683,7 +10653,7 @@
         <v/>
       </c>
     </row>
-    <row r="138" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="138" spans="8:31">
       <c r="H138" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Mechanical  - Screws</v>
@@ -10751,7 +10721,7 @@
         <v/>
       </c>
     </row>
-    <row r="139" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="139" spans="8:31">
       <c r="H139" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Protection - Fuses</v>
@@ -10819,7 +10789,7 @@
         <v/>
       </c>
     </row>
-    <row r="140" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="140" spans="8:31">
       <c r="H140" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Protection - GDT</v>
@@ -10887,7 +10857,7 @@
         <v/>
       </c>
     </row>
-    <row r="141" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="141" spans="8:31">
       <c r="H141" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Protection - MOVs</v>
@@ -10955,7 +10925,7 @@
         <v/>
       </c>
     </row>
-    <row r="142" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="142" spans="8:31">
       <c r="H142" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Protection - TVS Diode</v>
@@ -11023,7 +10993,7 @@
         <v/>
       </c>
     </row>
-    <row r="143" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="143" spans="8:31">
       <c r="H143" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>PSUs - PCB Mount - DC-DC - Non-Isolated</v>
@@ -11097,7 +11067,7 @@
         <v/>
       </c>
     </row>
-    <row r="144" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="144" spans="8:31">
       <c r="H144" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>PSUs - Wall Wart</v>
@@ -11165,7 +11135,7 @@
         <v/>
       </c>
     </row>
-    <row r="145" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="145" spans="8:31">
       <c r="H145" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Resistors - Isolated Array</v>
@@ -11233,7 +11203,7 @@
         <v/>
       </c>
     </row>
-    <row r="146" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="146" spans="8:31">
       <c r="H146" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Resistors - Single - SMD</v>
@@ -11304,7 +11274,7 @@
         <v/>
       </c>
     </row>
-    <row r="147" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="147" spans="8:31">
       <c r="H147" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Switches - Push</v>
@@ -11318,22 +11288,22 @@
       <c r="P147" s="6" t="b">
         <v>1</v>
       </c>
-      <c r="Q147" s="30" t="b">
-        <v>1</v>
-      </c>
-      <c r="R147" s="30" t="b">
+      <c r="Q147" t="b">
+        <v>1</v>
+      </c>
+      <c r="R147" t="b">
         <v>1</v>
       </c>
       <c r="S147" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="T147" s="30" t="b">
-        <v>1</v>
-      </c>
-      <c r="U147" s="30" t="b">
-        <v>1</v>
-      </c>
-      <c r="V147" s="30" t="b">
+      <c r="T147" t="b">
+        <v>1</v>
+      </c>
+      <c r="U147" t="b">
+        <v>1</v>
+      </c>
+      <c r="V147" t="b">
         <v>1</v>
       </c>
       <c r="W147">
@@ -11372,7 +11342,7 @@
         <v/>
       </c>
     </row>
-    <row r="148" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="148" spans="8:31">
       <c r="H148" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Switches - Slide</v>
@@ -11440,7 +11410,7 @@
         <v/>
       </c>
     </row>
-    <row r="149" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="149" spans="8:31">
       <c r="H149" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Switches - Tactile</v>
@@ -11508,7 +11478,7 @@
         <v/>
       </c>
     </row>
-    <row r="150" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="150" spans="8:31">
       <c r="H150" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Thermal - Heat Sinks</v>
@@ -11576,7 +11546,7 @@
         <v/>
       </c>
     </row>
-    <row r="151" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="151" spans="8:31">
       <c r="H151" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Thermal - Pads</v>
@@ -11644,7 +11614,7 @@
         <v/>
       </c>
     </row>
-    <row r="152" spans="8:31" x14ac:dyDescent="0.35">
+    <row r="152" spans="8:31">
       <c r="H152" t="str">
         <f>_xlfn.CONCAT(Table1[[#This Row],[Eff pt 1]:[Eff pt 7]])</f>
         <v>Voltage References - Burried Zener</v>
@@ -11726,31 +11696,31 @@
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="E15">
-    <cfRule type="cellIs" dxfId="9" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="5" priority="3" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H12:H152">
-    <cfRule type="expression" dxfId="8" priority="2">
+    <cfRule type="expression" dxfId="4" priority="2">
       <formula>IF($W12 = -1, 1, 0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H12:O9999">
-    <cfRule type="expression" dxfId="7" priority="36">
+    <cfRule type="expression" dxfId="3" priority="36">
       <formula>IF($W12 &gt;= $E$18, 1, 0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P12:V152">
-    <cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="TRALSE">
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="TRALSE">
       <formula>NOT(ISERROR(SEARCH("TRALSE",P12)))</formula>
     </cfRule>
     <cfRule type="containsBlanks" priority="5" stopIfTrue="1">
       <formula>LEN(TRIM(P12))=0</formula>
     </cfRule>
-    <cfRule type="notContainsText" dxfId="5" priority="6" operator="notContains" text="TRUE">
+    <cfRule type="notContainsText" dxfId="1" priority="6" operator="notContains" text="TRUE">
       <formula>ISERROR(SEARCH("TRUE",P12))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="7" operator="containsText" text="TRUE">
+    <cfRule type="containsText" dxfId="0" priority="7" operator="containsText" text="TRUE">
       <formula>NOT(ISERROR(SEARCH("TRUE",P12)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>